<commit_message>
fixed errors in inputData for calculation
</commit_message>
<xml_diff>
--- a/src/presentation/CielaDocs.SjcWeb/wwwroot/templates/AppCourtsCheck.xlsx
+++ b/src/presentation/CielaDocs.SjcWeb/wwwroot/templates/AppCourtsCheck.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\CielaTeams\VSS\SJCBProgs\src\presentation\CielaDocs.SjcWeb\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87F46AF3-0FCE-4387-B722-F1CD92DD4B52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BA17044-025C-4F46-93F0-D514B8C74B32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2652" yWindow="1452" windowWidth="27372" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="21900" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -25,12 +25,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>Справка за въведени данни от отчетни единици</t>
   </si>
   <si>
     <t>Отчетна единица</t>
+  </si>
+  <si>
+    <t>Статус</t>
   </si>
 </sst>
 </file>
@@ -96,19 +99,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -390,55 +385,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:H5"/>
+  <dimension ref="C2:D5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="3" max="3" width="71.77734375" customWidth="1"/>
+    <col min="4" max="4" width="23.77734375" customWidth="1"/>
     <col min="8" max="8" width="17.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B2" s="2" t="s">
+    <row r="2" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="2"/>
       <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
     </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-    </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B4" s="1"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-    </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="C5" s="3" t="s">
+    <row r="5" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C5" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
+      <c r="D5" s="1" t="s">
+        <v>2</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="B2:H2"/>
-    <mergeCell ref="C5:G5"/>
-    <mergeCell ref="C4:H4"/>
+  <mergeCells count="1">
+    <mergeCell ref="C2:D2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>